<commit_message>
Improve workbook export by sanitizing formula results
Introduce a `setFormula` helper function to sanitize and safely set formula values in the Excel export, preventing parsing errors caused by invalid number formats like NaN or Infinity.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a1e7a024-8deb-4e05-bb93-350fde674463
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: fcfe66fc-3bd3-4c27-9551-667fa70d8184
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/27fdbaf7-67db-442f-83d4-bebcb570d0b5/a1e7a024-8deb-4e05-bb93-350fde674463/vniIcGX
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/school-financial-model/public/proof_workbook.xlsx
+++ b/artifacts/school-financial-model/public/proof_workbook.xlsx
@@ -1575,23 +1575,23 @@
       </c>
       <c r="B8" s="11">
         <f>IF(B2=0,0,B7/B2)</f>
-        <v>-0.1898531902879729</v>
+        <v>-0.19</v>
       </c>
       <c r="C8" s="11">
         <f>IF(C2=0,0,C7/C2)</f>
-        <v>-0.0394026226323458</v>
+        <v>-0.04</v>
       </c>
       <c r="D8" s="11">
         <f>IF(D2=0,0,D7/D2)</f>
-        <v>0.10120486899112853</v>
+        <v>0.1</v>
       </c>
       <c r="E8" s="11">
         <f>IF(E2=0,0,E7/E2)</f>
-        <v>0.23371465051676243</v>
+        <v>0.23</v>
       </c>
       <c r="F8" s="11">
         <f>IF(F2=0,0,F7/F2)</f>
-        <v>0.3352791134044799</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1995,23 +1995,23 @@
       </c>
       <c r="B5" s="24">
         <f>IF(B4=0,"N/A",B3/B4)</f>
-        <v>-1.7966397737669466</v>
+        <v>-1.8</v>
       </c>
       <c r="C5" s="24">
         <f>IF(C4=0,"N/A",C3/C4)</f>
-        <v>0.3251268402229061</v>
+        <v>0.33</v>
       </c>
       <c r="D5" s="24">
         <f>IF(D4=0,"N/A",D3/D4)</f>
-        <v>3.039923479996673</v>
+        <v>3.04</v>
       </c>
       <c r="E5" s="24">
         <f>IF(E4=0,"N/A",E3/E4)</f>
-        <v>6.633036679697247</v>
+        <v>6.63</v>
       </c>
       <c r="F5" s="24">
         <f>IF(F4=0,"N/A",F3/F4)</f>
-        <v>10.511436413540714</v>
+        <v>10.51</v>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -2070,23 +2070,23 @@
       </c>
       <c r="B10" s="25">
         <f>IF(B9=0,0,B8/B9)</f>
-        <v>0.9890687281072593</v>
+        <v>0.99</v>
       </c>
       <c r="C10" s="25">
         <f>IF(C9=0,0,C8/C9)</f>
-        <v>0.4909404146616765</v>
+        <v>0.49</v>
       </c>
       <c r="D10" s="25">
         <f>IF(D9=0,0,D8/D9)</f>
-        <v>1.9120116618075802</v>
+        <v>1.91</v>
       </c>
       <c r="E10" s="25">
         <f>IF(E9=0,0,E8/E9)</f>
-        <v>5.74290121693424</v>
+        <v>5.74</v>
       </c>
       <c r="F10" s="25">
         <f>IF(F9=0,0,F8/F9)</f>
-        <v>12.009557344064387</v>
+        <v>12.01</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -2804,19 +2804,19 @@
       </c>
       <c r="C3" s="11">
         <f>IF(B2=0,"—",(C2-B2)/B2)</f>
-        <v>0.2222222222222222</v>
+        <v>0.22</v>
       </c>
       <c r="D3" s="11">
         <f>IF(C2=0,"—",(D2-C2)/C2)</f>
-        <v>0.18181818181818182</v>
+        <v>0.18</v>
       </c>
       <c r="E3" s="11">
         <f>IF(D2=0,"—",(E2-D2)/D2)</f>
-        <v>0.19230769230769232</v>
+        <v>0.19</v>
       </c>
       <c r="F3" s="11">
         <f>IF(E2=0,"—",(F2-E2)/E2)</f>
-        <v>0.16129032258064516</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>